<commit_message>
fix: corrections display names ValueSets (typos et harmonisation CodeSystems)
- FRCoreValueSetOrganizationType : "Pole" → "Pôle", "Groupe privé / hospitalier" → sans espaces
- FRCoreValueSetOrganizationIdentifierType : RPPSRG "Identifiant RPPS Rang" → "N° RPPS Rang", IDNST ASIP-SANTE → ANS
- FRCoreValueSetEncounterClass : NONAC "Inpatient non acute" → "inpatient non-acute"

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> 32e81051dbeed863c4906d623c23b7c0f0190564
</commit_message>
<xml_diff>
--- a/nr-add-more-examples/ig/ValueSet-fr-core-vs-encounter-class.xlsx
+++ b/nr-add-more-examples/ig/ValueSet-fr-core-vs-encounter-class.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-30T13:20:47+00:00</t>
+    <t>2026-04-30T13:24:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -114,7 +114,7 @@
     <t>NONAC</t>
   </si>
   <si>
-    <t>Inpatient non acute</t>
+    <t>inpatient non-acute</t>
   </si>
   <si>
     <t>PRENC</t>

</xml_diff>